<commit_message>
Updated Sectors.xlsx to work
</commit_message>
<xml_diff>
--- a/inst/extdata/sectors.xlsx
+++ b/inst/extdata/sectors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MinnaarC.EC_ATLANTIC\Desktop\POE\CWS-Pathway-of-Effects\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7773517B-4433-4658-922C-45F7AA7CB3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD93A2AA-A7E0-43C3-BA18-D0B9071CA7D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9555" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="58">
   <si>
     <t>Description</t>
   </si>
@@ -166,9 +166,6 @@
     <t>Vessels / shipping</t>
   </si>
   <si>
-    <t>Organic waste management and non-hazardous waste incineration</t>
-  </si>
-  <si>
     <t>Offshore Oil, Gas and other Fossil Fuels</t>
   </si>
   <si>
@@ -191,12 +188,6 @@
   </si>
   <si>
     <t>Aquaculture facility</t>
-  </si>
-  <si>
-    <t>Excavation and grading (e.g. site preparation, borrow pits, water management ponds,  diversion or drainage channels)</t>
-  </si>
-  <si>
-    <t>Linear right of way(s)  (e.g. transmission/distribution lines, pipelines, terrestrial seismic lines/mining exploration, roads)</t>
   </si>
   <si>
     <t>Renewable Energy – Land based Wind Power</t>
@@ -286,15 +277,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,10 +498,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="31.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
+      <c r="B2" s="12"/>
     </row>
     <row r="3" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -519,22 +510,22 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="9"/>
+      <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="9"/>
+      <c r="B6" s="12"/>
     </row>
     <row r="7" spans="1:2" ht="21.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="9"/>
+      <c r="B7" s="12"/>
     </row>
     <row r="8" spans="1:2" ht="21.65" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -543,10 +534,10 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="9"/>
+      <c r="B10" s="12"/>
     </row>
     <row r="11" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -555,10 +546,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9"/>
+      <c r="B13" s="12"/>
     </row>
     <row r="14" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="15" spans="1:2" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -642,8 +633,8 @@
       <c r="C1"/>
     </row>
     <row r="2" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
-        <v>50</v>
+      <c r="A2" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -651,8 +642,8 @@
       <c r="C2"/>
     </row>
     <row r="3" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
-        <v>50</v>
+      <c r="A3" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -660,8 +651,8 @@
       <c r="C3"/>
     </row>
     <row r="4" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>50</v>
+      <c r="A4" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>25</v>
@@ -669,8 +660,8 @@
       <c r="C4"/>
     </row>
     <row r="5" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>50</v>
+      <c r="A5" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>29</v>
@@ -678,8 +669,8 @@
       <c r="C5"/>
     </row>
     <row r="6" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
-        <v>50</v>
+      <c r="A6" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>12</v>
@@ -687,8 +678,8 @@
       <c r="C6"/>
     </row>
     <row r="7" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
-        <v>50</v>
+      <c r="A7" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>27</v>
@@ -696,8 +687,8 @@
       <c r="C7"/>
     </row>
     <row r="8" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
-        <v>50</v>
+      <c r="A8" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>37</v>
@@ -705,8 +696,8 @@
       <c r="C8"/>
     </row>
     <row r="9" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
-        <v>50</v>
+      <c r="A9" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>33</v>
@@ -714,8 +705,8 @@
       <c r="C9"/>
     </row>
     <row r="10" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
-        <v>50</v>
+      <c r="A10" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>24</v>
@@ -723,8 +714,8 @@
       <c r="C10"/>
     </row>
     <row r="11" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
-        <v>50</v>
+      <c r="A11" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>26</v>
@@ -732,8 +723,8 @@
       <c r="C11"/>
     </row>
     <row r="12" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="11" t="s">
-        <v>50</v>
+      <c r="A12" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>30</v>
@@ -741,17 +732,17 @@
       <c r="C12"/>
     </row>
     <row r="13" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
-        <v>50</v>
+      <c r="A13" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C13"/>
     </row>
     <row r="14" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="11" t="s">
-        <v>50</v>
+      <c r="A14" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>36</v>
@@ -759,116 +750,116 @@
       <c r="C14"/>
     </row>
     <row r="15" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="A15" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C15"/>
     </row>
     <row r="16" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="A16" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C16"/>
     </row>
     <row r="17" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>55</v>
+      <c r="A17" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C17"/>
     </row>
     <row r="18" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>25</v>
       </c>
       <c r="C18"/>
     </row>
     <row r="19" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>56</v>
+      <c r="A19" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="C19"/>
     </row>
     <row r="20" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="A20" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>12</v>
       </c>
       <c r="C20"/>
     </row>
     <row r="21" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="10" t="s">
+      <c r="A21" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>27</v>
       </c>
       <c r="C21"/>
     </row>
     <row r="22" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="12" t="s">
+      <c r="A22" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>35</v>
       </c>
       <c r="C22"/>
     </row>
     <row r="23" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>52</v>
+      <c r="A23" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="C23"/>
     </row>
     <row r="24" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="A24" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C24"/>
     </row>
     <row r="25" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="12" t="s">
+      <c r="A25" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C25"/>
     </row>
     <row r="26" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="A26" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>26</v>
       </c>
       <c r="C26"/>
     </row>
     <row r="27" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
-        <v>54</v>
+      <c r="A27" s="10" t="s">
+        <v>53</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>30</v>
@@ -876,17 +867,17 @@
       <c r="C27"/>
     </row>
     <row r="28" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="11" t="s">
-        <v>54</v>
+      <c r="A28" s="10" t="s">
+        <v>53</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C28"/>
     </row>
     <row r="29" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="11" t="s">
-        <v>54</v>
+      <c r="A29" s="10" t="s">
+        <v>53</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>36</v>
@@ -894,8 +885,8 @@
       <c r="C29"/>
     </row>
     <row r="30" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="11" t="s">
-        <v>54</v>
+      <c r="A30" s="10" t="s">
+        <v>53</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>34</v>
@@ -903,116 +894,116 @@
       <c r="C30"/>
     </row>
     <row r="31" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B31" s="12" t="s">
+      <c r="A31" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>40</v>
       </c>
       <c r="C31"/>
     </row>
     <row r="32" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="10" t="s">
+      <c r="A32" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C32"/>
     </row>
     <row r="33" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="10" t="s">
+      <c r="A33" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C33"/>
     </row>
     <row r="34" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="10" t="s">
+      <c r="A34" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C34"/>
     </row>
     <row r="35" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>55</v>
+      <c r="A35" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="C35"/>
     </row>
     <row r="36" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B36" s="10" t="s">
+      <c r="A36" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="9" t="s">
         <v>25</v>
       </c>
       <c r="C36"/>
     </row>
     <row r="37" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="10" t="s">
+      <c r="A37" s="10" t="s">
         <v>56</v>
       </c>
+      <c r="B37" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="C37"/>
     </row>
     <row r="38" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B38" s="10" t="s">
+      <c r="A38" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="9" t="s">
         <v>27</v>
       </c>
       <c r="C38"/>
     </row>
     <row r="39" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>52</v>
+      <c r="A39" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="C39"/>
     </row>
     <row r="40" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="10" t="s">
+      <c r="A40" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C40"/>
     </row>
     <row r="41" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B41" s="12" t="s">
+      <c r="A41" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C41"/>
     </row>
     <row r="42" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B42" s="10" t="s">
+      <c r="A42" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="9" t="s">
         <v>26</v>
       </c>
       <c r="C42"/>
     </row>
     <row r="43" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="11" t="s">
-        <v>59</v>
+      <c r="A43" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>30</v>
@@ -1020,26 +1011,26 @@
       <c r="C43"/>
     </row>
     <row r="44" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="11" t="s">
-        <v>59</v>
+      <c r="A44" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C44"/>
     </row>
     <row r="45" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B45" s="12" t="s">
+      <c r="A45" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B45" s="11" t="s">
         <v>39</v>
       </c>
       <c r="C45"/>
     </row>
     <row r="46" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="11" t="s">
-        <v>53</v>
+      <c r="A46" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -1047,8 +1038,8 @@
       <c r="C46"/>
     </row>
     <row r="47" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="11" t="s">
-        <v>53</v>
+      <c r="A47" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B47" t="s">
         <v>13</v>
@@ -1056,8 +1047,8 @@
       <c r="C47"/>
     </row>
     <row r="48" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="11" t="s">
-        <v>53</v>
+      <c r="A48" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B48" s="7" t="s">
         <v>25</v>
@@ -1065,8 +1056,8 @@
       <c r="C48"/>
     </row>
     <row r="49" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="11" t="s">
-        <v>53</v>
+      <c r="A49" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>27</v>
@@ -1074,8 +1065,8 @@
       <c r="C49"/>
     </row>
     <row r="50" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="11" t="s">
-        <v>53</v>
+      <c r="A50" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>35</v>
@@ -1083,8 +1074,8 @@
       <c r="C50"/>
     </row>
     <row r="51" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="11" t="s">
-        <v>53</v>
+      <c r="A51" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>37</v>
@@ -1092,8 +1083,8 @@
       <c r="C51"/>
     </row>
     <row r="52" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="11" t="s">
-        <v>53</v>
+      <c r="A52" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>33</v>
@@ -1101,17 +1092,17 @@
       <c r="C52"/>
     </row>
     <row r="53" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B53" s="12" t="s">
+      <c r="A53" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C53"/>
     </row>
     <row r="54" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="11" t="s">
-        <v>53</v>
+      <c r="A54" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B54" s="7" t="s">
         <v>30</v>
@@ -1119,17 +1110,17 @@
       <c r="C54"/>
     </row>
     <row r="55" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="11" t="s">
-        <v>53</v>
+      <c r="A55" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C55"/>
     </row>
     <row r="56" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="11" t="s">
-        <v>53</v>
+      <c r="A56" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B56" s="7" t="s">
         <v>36</v>
@@ -1137,8 +1128,8 @@
       <c r="C56"/>
     </row>
     <row r="57" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="11" t="s">
-        <v>53</v>
+      <c r="A57" s="10" t="s">
+        <v>52</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>34</v>
@@ -1146,55 +1137,55 @@
       <c r="C57"/>
     </row>
     <row r="58" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B58" s="10" t="s">
+      <c r="A58" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B58" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C58"/>
     </row>
     <row r="59" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B59" s="10" t="s">
+      <c r="A59" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B59" s="9" t="s">
         <v>40</v>
       </c>
       <c r="C59"/>
     </row>
     <row r="60" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B60" s="10" t="s">
+      <c r="A60" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C60"/>
     </row>
     <row r="61" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B61" s="10" t="s">
+      <c r="A61" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C61"/>
     </row>
     <row r="62" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B62" s="10" t="s">
+      <c r="A62" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B62" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C62"/>
     </row>
     <row r="63" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B63" s="10" t="s">
+      <c r="A63" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B63" s="9" t="s">
         <v>45</v>
       </c>
       <c r="C63"/>
@@ -1300,7 +1291,7 @@
         <v>15</v>
       </c>
       <c r="B76" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.35">
@@ -1444,7 +1435,7 @@
         <v>16</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.35">
@@ -1580,7 +1571,7 @@
         <v>17</v>
       </c>
       <c r="B111" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.35">
@@ -1593,87 +1584,87 @@
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B113" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B113" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B114" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
+      </c>
+      <c r="B114" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B115" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B115" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B116" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="B116" s="9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B117" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B117" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B118" s="10" t="s">
-        <v>52</v>
+        <v>57</v>
+      </c>
+      <c r="B118" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B119" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B119" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B120" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B120" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B121" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B121" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B122" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B122" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B123" s="7" t="s">
         <v>30</v>
@@ -1681,23 +1672,23 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B125" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B125" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B126" t="s">
         <v>14</v>
@@ -1705,7 +1696,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B127" t="s">
         <v>13</v>
@@ -1713,7 +1704,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B128" s="7" t="s">
         <v>25</v>
@@ -1721,7 +1712,7 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B129" s="7" t="s">
         <v>29</v>
@@ -1729,7 +1720,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B130" s="7" t="s">
         <v>12</v>
@@ -1737,7 +1728,7 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B131" s="7" t="s">
         <v>27</v>
@@ -1745,7 +1736,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B132" s="7" t="s">
         <v>35</v>
@@ -1753,7 +1744,7 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B133" s="7" t="s">
         <v>37</v>
@@ -1761,7 +1752,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B134" s="7" t="s">
         <v>33</v>
@@ -1769,7 +1760,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B135" s="7" t="s">
         <v>24</v>
@@ -1777,7 +1768,7 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B136" s="7" t="s">
         <v>26</v>
@@ -1785,7 +1776,7 @@
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B137" s="7" t="s">
         <v>30</v>
@@ -1793,15 +1784,15 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B138" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B139" s="7" t="s">
         <v>36</v>
@@ -1809,7 +1800,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B140" s="7" t="s">
         <v>34</v>
@@ -1817,7 +1808,7 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B141" t="s">
         <v>38</v>
@@ -1825,7 +1816,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>28</v>
@@ -1833,7 +1824,7 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>32</v>
@@ -1841,7 +1832,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>45</v>
@@ -1849,7 +1840,7 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>14</v>
@@ -1857,7 +1848,7 @@
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>13</v>
@@ -1865,7 +1856,7 @@
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>25</v>
@@ -1873,7 +1864,7 @@
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>29</v>
@@ -1881,7 +1872,7 @@
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>12</v>
@@ -1889,7 +1880,7 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>27</v>
@@ -1897,39 +1888,39 @@
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
+        <v>50</v>
+      </c>
+      <c r="B151" s="9" t="s">
         <v>51</v>
-      </c>
-      <c r="B151" s="10" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>51</v>
-      </c>
-      <c r="B152" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B152" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>51</v>
-      </c>
-      <c r="B153" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B153" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>51</v>
-      </c>
-      <c r="B154" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B154" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>30</v>
@@ -1937,15 +1928,15 @@
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B156" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>36</v>
@@ -2076,7 +2067,7 @@
         <v>18</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.35">
@@ -2228,7 +2219,7 @@
         <v>19</v>
       </c>
       <c r="B192" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.35">
@@ -2388,7 +2379,7 @@
         <v>20</v>
       </c>
       <c r="B212" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.35">
@@ -2457,7 +2448,7 @@
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B221" t="s">
         <v>27</v>
@@ -2465,7 +2456,7 @@
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B222" t="s">
         <v>35</v>
@@ -2473,7 +2464,7 @@
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B223" t="s">
         <v>37</v>
@@ -2481,7 +2472,7 @@
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B224" t="s">
         <v>33</v>
@@ -2489,7 +2480,7 @@
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B225" s="7" t="s">
         <v>43</v>
@@ -2497,7 +2488,7 @@
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B226" s="7" t="s">
         <v>24</v>
@@ -2505,7 +2496,7 @@
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B227" s="7" t="s">
         <v>26</v>
@@ -2513,7 +2504,7 @@
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B228" s="7" t="s">
         <v>30</v>
@@ -2521,15 +2512,15 @@
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B229" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B230" s="7" t="s">
         <v>36</v>
@@ -2537,7 +2528,7 @@
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B231" s="7" t="s">
         <v>34</v>
@@ -2545,7 +2536,7 @@
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B232" s="7" t="s">
         <v>44</v>
@@ -2553,7 +2544,7 @@
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B233" s="7" t="s">
         <v>32</v>
@@ -2561,7 +2552,7 @@
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B234" s="7" t="s">
         <v>45</v>
@@ -2676,7 +2667,7 @@
         <v>21</v>
       </c>
       <c r="B248" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.35">
@@ -2737,7 +2728,7 @@
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B256" t="s">
         <v>14</v>
@@ -2745,7 +2736,7 @@
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B257" t="s">
         <v>13</v>
@@ -2753,7 +2744,7 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B258" t="s">
         <v>25</v>
@@ -2761,7 +2752,7 @@
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B259" t="s">
         <v>29</v>
@@ -2769,39 +2760,39 @@
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>57</v>
-      </c>
-      <c r="B260" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B260" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>57</v>
-      </c>
-      <c r="B261" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B261" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>57</v>
-      </c>
-      <c r="B262" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="B262" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>57</v>
-      </c>
-      <c r="B263" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B263" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B264" s="7" t="s">
         <v>24</v>
@@ -2809,15 +2800,15 @@
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>57</v>
-      </c>
-      <c r="B265" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B265" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B266" s="7" t="s">
         <v>41</v>
@@ -2825,7 +2816,7 @@
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B267" s="7" t="s">
         <v>30</v>
@@ -2833,15 +2824,15 @@
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B268" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B269" s="7" t="s">
         <v>36</v>
@@ -2849,7 +2840,7 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B270" s="7" t="s">
         <v>34</v>
@@ -2857,47 +2848,47 @@
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>57</v>
-      </c>
-      <c r="B271" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B271" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>57</v>
-      </c>
-      <c r="B272" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B272" s="11" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>57</v>
-      </c>
-      <c r="B273" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B273" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>57</v>
-      </c>
-      <c r="B274" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B274" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>57</v>
-      </c>
-      <c r="B275" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B275" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B276" s="7" t="s">
         <v>27</v>
@@ -2905,7 +2896,7 @@
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B277" s="8" t="s">
         <v>35</v>
@@ -2913,7 +2904,7 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B278" s="7" t="s">
         <v>37</v>
@@ -2921,7 +2912,7 @@
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B279" s="7" t="s">
         <v>33</v>
@@ -2929,7 +2920,7 @@
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B280" s="7" t="s">
         <v>24</v>
@@ -2937,7 +2928,7 @@
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B281" s="7" t="s">
         <v>26</v>
@@ -2945,7 +2936,7 @@
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B282" s="7" t="s">
         <v>30</v>
@@ -2953,15 +2944,15 @@
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B283" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B284" s="7" t="s">
         <v>36</v>
@@ -2969,7 +2960,7 @@
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B285" s="7" t="s">
         <v>34</v>
@@ -2977,7 +2968,7 @@
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B286" s="7" t="s">
         <v>44</v>
@@ -2985,7 +2976,7 @@
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B287" s="7" t="s">
         <v>32</v>
@@ -2993,7 +2984,7 @@
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B288" s="7" t="s">
         <v>45</v>
@@ -3100,7 +3091,7 @@
         <v>22</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.35">
@@ -3145,63 +3136,63 @@
     </row>
     <row r="307" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>58</v>
-      </c>
-      <c r="B307" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B307" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="308" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>58</v>
-      </c>
-      <c r="B308" s="10" t="s">
         <v>55</v>
+      </c>
+      <c r="B308" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="309" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>58</v>
-      </c>
-      <c r="B309" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="B309" s="9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="310" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>58</v>
-      </c>
-      <c r="B310" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B310" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="311" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>58</v>
-      </c>
-      <c r="B311" s="10" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="B311" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="312" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>58</v>
-      </c>
-      <c r="B312" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B312" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>58</v>
-      </c>
-      <c r="B313" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B313" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="314" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B314" s="7" t="s">
         <v>41</v>
@@ -3209,7 +3200,7 @@
     </row>
     <row r="315" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B315" s="7" t="s">
         <v>30</v>
@@ -3217,15 +3208,15 @@
     </row>
     <row r="316" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B316" s="7" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="317" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B317" s="7" t="s">
         <v>36</v>
@@ -3233,7 +3224,7 @@
     </row>
     <row r="318" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B318" s="7" t="s">
         <v>34</v>
@@ -3241,33 +3232,33 @@
     </row>
     <row r="319" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>58</v>
-      </c>
-      <c r="B319" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B319" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="320" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
-        <v>58</v>
-      </c>
-      <c r="B320" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B320" s="11" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="321" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
-        <v>58</v>
-      </c>
-      <c r="B321" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B321" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="322" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>58</v>
-      </c>
-      <c r="B322" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B322" s="9" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>